<commit_message>
Add end-to-end Appium CI workflow with Excel reporting
</commit_message>
<xml_diff>
--- a/appium_tests/reports/pytest_appium_results.xlsx
+++ b/appium_tests/reports/pytest_appium_results.xlsx
@@ -427,7 +427,7 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -464,7 +464,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test_generate_report</t>
+          <t>test_generate_excel_report</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -478,7 +478,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-02T22:26:57</t>
+          <t>2026-08-02T22:41:01</t>
         </is>
       </c>
     </row>

</xml_diff>